<commit_message>
punch display ui changes
</commit_message>
<xml_diff>
--- a/server/BIOMETRICEMPLOYEE.xlsx
+++ b/server/BIOMETRICEMPLOYEE.xlsx
@@ -1,33 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20417"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\ML Cabigas\dmbbhr\server\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D81C9A07-AB26-422B-82C1-E872A39FCD48}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="7800"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7395" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="181029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="174">
   <si>
     <t>ID</t>
   </si>
@@ -546,20 +539,19 @@
   </si>
   <si>
     <t>Abalo, Oliver</t>
+  </si>
+  <si>
+    <t>Cabalan, Janrey</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="5">
-    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="42" formatCode="_-&quot;₱&quot;* #,##0_-;\-&quot;₱&quot;* #,##0_-;_-&quot;₱&quot;* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="44" formatCode="_-&quot;₱&quot;* #,##0.00_-;\-&quot;₱&quot;* #,##0.00_-;_-&quot;₱&quot;* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="176" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -616,353 +608,16 @@
       <charset val="134"/>
       <scheme val="major"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="33">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -970,251 +625,9 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -1226,68 +639,24 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Link" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1485,24 +854,25 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:F148"/>
-  <sheetFormatPr defaultColWidth="12.5740740740741" defaultRowHeight="15.75" customHeight="1" outlineLevelCol="5"/>
+  <dimension ref="A1:F149"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="2" max="2" width="20.8518518518519" customWidth="1"/>
-    <col min="3" max="3" width="14.4259259259259" customWidth="1"/>
-    <col min="4" max="4" width="19.5740740740741" customWidth="1"/>
-    <col min="5" max="5" width="16.8518518518519" style="1" customWidth="1"/>
+    <col min="2" max="2" width="20.85546875" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" customWidth="1"/>
+    <col min="4" max="4" width="19.5703125" customWidth="1"/>
+    <col min="5" max="5" width="16.85546875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:6">
+    <row r="1" spans="1:6" ht="15.75" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1522,7 +892,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" customHeight="1" spans="1:6">
+    <row r="2" spans="1:6" ht="15.75" customHeight="1">
       <c r="A2" s="5">
         <v>25069</v>
       </c>
@@ -1536,7 +906,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" customHeight="1" spans="1:6">
+    <row r="3" spans="1:6" ht="15.75" customHeight="1">
       <c r="A3" s="5">
         <v>50008</v>
       </c>
@@ -1550,7 +920,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" customHeight="1" spans="1:6">
+    <row r="4" spans="1:6" ht="15.75" customHeight="1">
       <c r="A4" s="5">
         <v>50046</v>
       </c>
@@ -1564,7 +934,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" customHeight="1" spans="1:6">
+    <row r="5" spans="1:6" ht="15.75" customHeight="1">
       <c r="A5" s="5">
         <v>50048</v>
       </c>
@@ -1578,7 +948,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" customHeight="1" spans="1:6">
+    <row r="6" spans="1:6" ht="15.75" customHeight="1">
       <c r="A6" s="5">
         <v>50071</v>
       </c>
@@ -1592,7 +962,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" customHeight="1" spans="1:6">
+    <row r="7" spans="1:6" ht="15.75" customHeight="1">
       <c r="A7" s="5">
         <v>50113</v>
       </c>
@@ -1606,7 +976,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" customHeight="1" spans="1:6">
+    <row r="8" spans="1:6" ht="15.75" customHeight="1">
       <c r="A8" s="5">
         <v>50190</v>
       </c>
@@ -1620,7 +990,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" customHeight="1" spans="1:6">
+    <row r="9" spans="1:6" ht="15.75" customHeight="1">
       <c r="A9" s="5">
         <v>25041</v>
       </c>
@@ -1634,7 +1004,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" customHeight="1" spans="1:6">
+    <row r="10" spans="1:6" ht="15.75" customHeight="1">
       <c r="A10" s="5">
         <v>25065</v>
       </c>
@@ -1648,7 +1018,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" customHeight="1" spans="1:6">
+    <row r="11" spans="1:6" ht="15.75" customHeight="1">
       <c r="A11" s="5">
         <v>50329</v>
       </c>
@@ -1662,7 +1032,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" customHeight="1" spans="1:6">
+    <row r="12" spans="1:6" ht="15.75" customHeight="1">
       <c r="A12" s="5">
         <v>50336</v>
       </c>
@@ -1676,7 +1046,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" customHeight="1" spans="1:6">
+    <row r="13" spans="1:6" ht="15.75" customHeight="1">
       <c r="A13" s="5">
         <v>58337</v>
       </c>
@@ -1690,7 +1060,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="14" customHeight="1" spans="1:6">
+    <row r="14" spans="1:6" ht="15.75" customHeight="1">
       <c r="A14" s="5">
         <v>25001</v>
       </c>
@@ -1704,7 +1074,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" customHeight="1" spans="1:6">
+    <row r="15" spans="1:6" ht="15.75" customHeight="1">
       <c r="A15" s="5">
         <v>25003</v>
       </c>
@@ -1718,7 +1088,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" customHeight="1" spans="1:6">
+    <row r="16" spans="1:6" ht="15.75" customHeight="1">
       <c r="A16" s="5">
         <v>25021</v>
       </c>
@@ -1732,7 +1102,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" customHeight="1" spans="1:6">
+    <row r="17" spans="1:6" ht="15.75" customHeight="1">
       <c r="A17" s="5">
         <v>25024</v>
       </c>
@@ -1746,7 +1116,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" customHeight="1" spans="1:6">
+    <row r="18" spans="1:6" ht="15.75" customHeight="1">
       <c r="A18" s="5">
         <v>25025</v>
       </c>
@@ -1760,7 +1130,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" customHeight="1" spans="1:6">
+    <row r="19" spans="1:6" ht="15.75" customHeight="1">
       <c r="A19" s="5">
         <v>25027</v>
       </c>
@@ -1774,7 +1144,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" customHeight="1" spans="1:6">
+    <row r="20" spans="1:6" ht="15.75" customHeight="1">
       <c r="A20" s="5">
         <v>25032</v>
       </c>
@@ -1788,7 +1158,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="21" customHeight="1" spans="1:6">
+    <row r="21" spans="1:6" ht="15.75" customHeight="1">
       <c r="A21" s="5">
         <v>25034</v>
       </c>
@@ -1802,7 +1172,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" customHeight="1" spans="1:6">
+    <row r="22" spans="1:6" ht="15.75" customHeight="1">
       <c r="A22" s="5">
         <v>25036</v>
       </c>
@@ -1816,7 +1186,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" customHeight="1" spans="1:6">
+    <row r="23" spans="1:6" ht="15.75" customHeight="1">
       <c r="A23" s="5">
         <v>25037</v>
       </c>
@@ -1830,7 +1200,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="24" customHeight="1" spans="1:6">
+    <row r="24" spans="1:6" ht="15.75" customHeight="1">
       <c r="A24" s="5">
         <v>25042</v>
       </c>
@@ -1844,7 +1214,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" customHeight="1" spans="1:6">
+    <row r="25" spans="1:6" ht="15.75" customHeight="1">
       <c r="A25" s="5">
         <v>25043</v>
       </c>
@@ -1858,7 +1228,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" customHeight="1" spans="1:6">
+    <row r="26" spans="1:6" ht="15.75" customHeight="1">
       <c r="A26" s="5">
         <v>25044</v>
       </c>
@@ -1872,7 +1242,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="27" customHeight="1" spans="1:6">
+    <row r="27" spans="1:6" ht="15.75" customHeight="1">
       <c r="A27" s="5">
         <v>25045</v>
       </c>
@@ -1886,7 +1256,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" customHeight="1" spans="1:6">
+    <row r="28" spans="1:6" ht="15.75" customHeight="1">
       <c r="A28" s="5">
         <v>25046</v>
       </c>
@@ -1900,7 +1270,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="29" customHeight="1" spans="1:6">
+    <row r="29" spans="1:6" ht="15.75" customHeight="1">
       <c r="A29" s="5">
         <v>25050</v>
       </c>
@@ -1914,7 +1284,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="30" customHeight="1" spans="1:6">
+    <row r="30" spans="1:6" ht="15.75" customHeight="1">
       <c r="A30" s="5">
         <v>25054</v>
       </c>
@@ -1928,7 +1298,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" customHeight="1" spans="1:6">
+    <row r="31" spans="1:6" ht="15.75" customHeight="1">
       <c r="A31" s="5">
         <v>25058</v>
       </c>
@@ -1942,7 +1312,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="32" customHeight="1" spans="1:6">
+    <row r="32" spans="1:6" ht="15.75" customHeight="1">
       <c r="A32" s="5">
         <v>25059</v>
       </c>
@@ -1956,7 +1326,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="33" customHeight="1" spans="1:6">
+    <row r="33" spans="1:6" ht="15.75" customHeight="1">
       <c r="A33" s="5">
         <v>25062</v>
       </c>
@@ -1970,7 +1340,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="34" customHeight="1" spans="1:6">
+    <row r="34" spans="1:6" ht="15.75" customHeight="1">
       <c r="A34" s="5">
         <v>25063</v>
       </c>
@@ -1984,7 +1354,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="35" customHeight="1" spans="1:6">
+    <row r="35" spans="1:6" ht="15.75" customHeight="1">
       <c r="A35" s="5">
         <v>25068</v>
       </c>
@@ -1998,7 +1368,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="36" customHeight="1" spans="1:6">
+    <row r="36" spans="1:6" ht="15.75" customHeight="1">
       <c r="A36" s="5">
         <v>25070</v>
       </c>
@@ -2012,7 +1382,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="37" customHeight="1" spans="1:6">
+    <row r="37" spans="1:6" ht="15.75" customHeight="1">
       <c r="A37" s="5">
         <v>25071</v>
       </c>
@@ -2026,7 +1396,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="38" customHeight="1" spans="1:6">
+    <row r="38" spans="1:6" ht="15.75" customHeight="1">
       <c r="A38" s="5">
         <v>25072</v>
       </c>
@@ -2040,7 +1410,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="39" customHeight="1" spans="1:6">
+    <row r="39" spans="1:6" ht="15.75" customHeight="1">
       <c r="A39" s="5">
         <v>25073</v>
       </c>
@@ -2054,7 +1424,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="40" customHeight="1" spans="1:6">
+    <row r="40" spans="1:6" ht="15.75" customHeight="1">
       <c r="A40" s="5">
         <v>25074</v>
       </c>
@@ -2068,7 +1438,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="41" customHeight="1" spans="1:6">
+    <row r="41" spans="1:6" ht="15.75" customHeight="1">
       <c r="A41" s="5">
         <v>50059</v>
       </c>
@@ -2082,7 +1452,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="42" customHeight="1" spans="1:6">
+    <row r="42" spans="1:6" ht="15.75" customHeight="1">
       <c r="A42" s="5">
         <v>50189</v>
       </c>
@@ -2096,7 +1466,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="43" customHeight="1" spans="1:6">
+    <row r="43" spans="1:6" ht="15.75" customHeight="1">
       <c r="A43" s="5">
         <v>50350</v>
       </c>
@@ -2110,7 +1480,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="44" customHeight="1" spans="1:6">
+    <row r="44" spans="1:6" ht="15.75" customHeight="1">
       <c r="A44" s="5">
         <v>5021</v>
       </c>
@@ -2127,7 +1497,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="45" customHeight="1" spans="1:6">
+    <row r="45" spans="1:6" ht="15.75" customHeight="1">
       <c r="A45" s="5">
         <v>25017</v>
       </c>
@@ -2141,7 +1511,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="46" customHeight="1" spans="1:6">
+    <row r="46" spans="1:6" ht="15.75" customHeight="1">
       <c r="A46" s="5">
         <v>25028</v>
       </c>
@@ -2155,7 +1525,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="47" customHeight="1" spans="1:6">
+    <row r="47" spans="1:6" ht="15.75" customHeight="1">
       <c r="A47" s="5">
         <v>25031</v>
       </c>
@@ -2169,7 +1539,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="48" customHeight="1" spans="1:6">
+    <row r="48" spans="1:6" ht="15.75" customHeight="1">
       <c r="A48" s="5">
         <v>25039</v>
       </c>
@@ -2183,7 +1553,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="49" customHeight="1" spans="1:6">
+    <row r="49" spans="1:6" ht="15.75" customHeight="1">
       <c r="A49" s="5">
         <v>25040</v>
       </c>
@@ -2200,7 +1570,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="50" customHeight="1" spans="1:6">
+    <row r="50" spans="1:6" ht="15.75" customHeight="1">
       <c r="A50" s="5">
         <v>25053</v>
       </c>
@@ -2214,7 +1584,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="51" customHeight="1" spans="1:6">
+    <row r="51" spans="1:6" ht="15.75" customHeight="1">
       <c r="A51" s="5">
         <v>25060</v>
       </c>
@@ -2228,7 +1598,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="52" customHeight="1" spans="1:6">
+    <row r="52" spans="1:6" ht="15.75" customHeight="1">
       <c r="A52" s="5">
         <v>50007</v>
       </c>
@@ -2242,7 +1612,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="53" customHeight="1" spans="1:6">
+    <row r="53" spans="1:6" ht="15.75" customHeight="1">
       <c r="A53" s="5">
         <v>50014</v>
       </c>
@@ -2256,7 +1626,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="54" customHeight="1" spans="1:6">
+    <row r="54" spans="1:6" ht="15.75" customHeight="1">
       <c r="A54" s="5">
         <v>50015</v>
       </c>
@@ -2270,7 +1640,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="55" customHeight="1" spans="1:6">
+    <row r="55" spans="1:6" ht="15.75" customHeight="1">
       <c r="A55" s="5">
         <v>50016</v>
       </c>
@@ -2284,7 +1654,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="56" customHeight="1" spans="1:6">
+    <row r="56" spans="1:6" ht="15.75" customHeight="1">
       <c r="A56" s="5">
         <v>50017</v>
       </c>
@@ -2301,7 +1671,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="57" customHeight="1" spans="1:6">
+    <row r="57" spans="1:6" ht="15.75" customHeight="1">
       <c r="A57" s="5">
         <v>50018</v>
       </c>
@@ -2315,7 +1685,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="58" customHeight="1" spans="1:6">
+    <row r="58" spans="1:6" ht="15.75" customHeight="1">
       <c r="A58" s="5">
         <v>50020</v>
       </c>
@@ -2329,7 +1699,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="59" customHeight="1" spans="1:6">
+    <row r="59" spans="1:6" ht="15.75" customHeight="1">
       <c r="A59" s="5">
         <v>50026</v>
       </c>
@@ -2343,7 +1713,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="60" customHeight="1" spans="1:6">
+    <row r="60" spans="1:6" ht="15.75" customHeight="1">
       <c r="A60" s="5">
         <v>50140</v>
       </c>
@@ -2360,7 +1730,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="61" customHeight="1" spans="1:6">
+    <row r="61" spans="1:6" ht="15.75" customHeight="1">
       <c r="A61" s="5">
         <v>50160</v>
       </c>
@@ -2374,7 +1744,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="62" customHeight="1" spans="1:6">
+    <row r="62" spans="1:6" ht="15.75" customHeight="1">
       <c r="A62" s="5">
         <v>50253</v>
       </c>
@@ -2388,7 +1758,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="63" customHeight="1" spans="1:6">
+    <row r="63" spans="1:6" ht="15.75" customHeight="1">
       <c r="A63" s="5">
         <v>50347</v>
       </c>
@@ -2402,7 +1772,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="64" customHeight="1" spans="1:6">
+    <row r="64" spans="1:6" ht="15.75" customHeight="1">
       <c r="A64" s="5">
         <v>50351</v>
       </c>
@@ -2416,7 +1786,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="65" customHeight="1" spans="1:6">
+    <row r="65" spans="1:6" ht="15.75" customHeight="1">
       <c r="A65" s="5">
         <v>50363</v>
       </c>
@@ -2430,7 +1800,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="66" customHeight="1" spans="1:6">
+    <row r="66" spans="1:6" ht="15.75" customHeight="1">
       <c r="A66" s="5">
         <v>500386</v>
       </c>
@@ -2447,7 +1817,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="67" customHeight="1" spans="1:6">
+    <row r="67" spans="1:6" ht="15.75" customHeight="1">
       <c r="A67" s="5">
         <v>500387</v>
       </c>
@@ -2461,7 +1831,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="68" customHeight="1" spans="1:6">
+    <row r="68" spans="1:6" ht="15.75" customHeight="1">
       <c r="A68" s="5">
         <v>500388</v>
       </c>
@@ -2475,7 +1845,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="69" customHeight="1" spans="1:6">
+    <row r="69" spans="1:6" ht="15.75" customHeight="1">
       <c r="A69" s="5">
         <v>500389</v>
       </c>
@@ -2489,7 +1859,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="70" customHeight="1" spans="1:6">
+    <row r="70" spans="1:6" ht="15.75" customHeight="1">
       <c r="A70" s="5">
         <v>500390</v>
       </c>
@@ -2506,7 +1876,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="71" customHeight="1" spans="1:6">
+    <row r="71" spans="1:6" ht="15.75" customHeight="1">
       <c r="A71" s="5">
         <v>500391</v>
       </c>
@@ -2520,7 +1890,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="72" customHeight="1" spans="1:6">
+    <row r="72" spans="1:6" ht="15.75" customHeight="1">
       <c r="A72" s="5">
         <v>500392</v>
       </c>
@@ -2534,7 +1904,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="73" customHeight="1" spans="1:6">
+    <row r="73" spans="1:6" ht="15.75" customHeight="1">
       <c r="A73" s="5">
         <v>500393</v>
       </c>
@@ -2548,7 +1918,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="74" customHeight="1" spans="1:6">
+    <row r="74" spans="1:6" ht="15.75" customHeight="1">
       <c r="A74" s="5">
         <v>500394</v>
       </c>
@@ -2562,7 +1932,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="75" customHeight="1" spans="1:6">
+    <row r="75" spans="1:6" ht="15.75" customHeight="1">
       <c r="A75" s="5">
         <v>500395</v>
       </c>
@@ -2576,7 +1946,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="76" customHeight="1" spans="1:6">
+    <row r="76" spans="1:6" ht="15.75" customHeight="1">
       <c r="A76" s="5">
         <v>500396</v>
       </c>
@@ -2590,7 +1960,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="77" customHeight="1" spans="1:6">
+    <row r="77" spans="1:6" ht="15.75" customHeight="1">
       <c r="A77" s="5">
         <v>500397</v>
       </c>
@@ -2604,7 +1974,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="78" customHeight="1" spans="1:6">
+    <row r="78" spans="1:6" ht="15.75" customHeight="1">
       <c r="A78" s="5">
         <v>500398</v>
       </c>
@@ -2618,7 +1988,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="79" customHeight="1" spans="1:6">
+    <row r="79" spans="1:6" ht="15.75" customHeight="1">
       <c r="A79" s="5">
         <v>500399</v>
       </c>
@@ -2632,7 +2002,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="80" customHeight="1" spans="1:6">
+    <row r="80" spans="1:6" ht="15.75" customHeight="1">
       <c r="A80" s="5">
         <v>25005</v>
       </c>
@@ -2646,7 +2016,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="81" customHeight="1" spans="1:6">
+    <row r="81" spans="1:6" ht="15.75" customHeight="1">
       <c r="A81" s="5">
         <v>25013</v>
       </c>
@@ -2660,7 +2030,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="82" customHeight="1" spans="1:6">
+    <row r="82" spans="1:6" ht="15.75" customHeight="1">
       <c r="A82" s="5">
         <v>25019</v>
       </c>
@@ -2674,7 +2044,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="83" customHeight="1" spans="1:6">
+    <row r="83" spans="1:6" ht="15.75" customHeight="1">
       <c r="A83" s="5">
         <v>25057</v>
       </c>
@@ -2688,7 +2058,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="84" customHeight="1" spans="1:6">
+    <row r="84" spans="1:6" ht="15.75" customHeight="1">
       <c r="A84" s="5">
         <v>50030</v>
       </c>
@@ -2702,7 +2072,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="85" customHeight="1" spans="1:6">
+    <row r="85" spans="1:6" ht="15.75" customHeight="1">
       <c r="A85" s="5">
         <v>50031</v>
       </c>
@@ -2716,7 +2086,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="86" customHeight="1" spans="1:6">
+    <row r="86" spans="1:6" ht="15.75" customHeight="1">
       <c r="A86" s="5">
         <v>50038</v>
       </c>
@@ -2730,7 +2100,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="87" customHeight="1" spans="1:6">
+    <row r="87" spans="1:6" ht="15.75" customHeight="1">
       <c r="A87" s="5">
         <v>50039</v>
       </c>
@@ -2744,7 +2114,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="88" customHeight="1" spans="1:6">
+    <row r="88" spans="1:6" ht="15.75" customHeight="1">
       <c r="A88" s="5">
         <v>50050</v>
       </c>
@@ -2758,7 +2128,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="89" customHeight="1" spans="1:6">
+    <row r="89" spans="1:6" ht="15.75" customHeight="1">
       <c r="A89" s="5">
         <v>50060</v>
       </c>
@@ -2772,7 +2142,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="90" customHeight="1" spans="1:6">
+    <row r="90" spans="1:6" ht="15.75" customHeight="1">
       <c r="A90" s="5">
         <v>50062</v>
       </c>
@@ -2786,7 +2156,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="91" customHeight="1" spans="1:6">
+    <row r="91" spans="1:6" ht="15.75" customHeight="1">
       <c r="A91" s="5">
         <v>50065</v>
       </c>
@@ -2800,7 +2170,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="92" customHeight="1" spans="1:6">
+    <row r="92" spans="1:6" ht="15.75" customHeight="1">
       <c r="A92" s="5">
         <v>50099</v>
       </c>
@@ -2814,7 +2184,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="93" customHeight="1" spans="1:6">
+    <row r="93" spans="1:6" ht="15.75" customHeight="1">
       <c r="A93" s="5">
         <v>50218</v>
       </c>
@@ -2828,7 +2198,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="94" customHeight="1" spans="1:6">
+    <row r="94" spans="1:6" ht="15.75" customHeight="1">
       <c r="A94" s="5">
         <v>50245</v>
       </c>
@@ -2842,7 +2212,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="95" customHeight="1" spans="1:6">
+    <row r="95" spans="1:6" ht="15.75" customHeight="1">
       <c r="A95" s="5">
         <v>50263</v>
       </c>
@@ -2856,7 +2226,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="96" customHeight="1" spans="1:6">
+    <row r="96" spans="1:6" ht="15.75" customHeight="1">
       <c r="A96" s="5">
         <v>50281</v>
       </c>
@@ -2870,7 +2240,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="97" customHeight="1" spans="1:6">
+    <row r="97" spans="1:6" ht="15.75" customHeight="1">
       <c r="A97" s="5">
         <v>50294</v>
       </c>
@@ -2884,7 +2254,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="98" customHeight="1" spans="1:6">
+    <row r="98" spans="1:6" ht="15.75" customHeight="1">
       <c r="A98" s="5">
         <v>50323</v>
       </c>
@@ -2898,7 +2268,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="99" customHeight="1" spans="1:6">
+    <row r="99" spans="1:6" ht="15.75" customHeight="1">
       <c r="A99" s="5">
         <v>50341</v>
       </c>
@@ -2912,7 +2282,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="100" customHeight="1" spans="1:6">
+    <row r="100" spans="1:6" ht="15.75" customHeight="1">
       <c r="A100" s="5">
         <v>50343</v>
       </c>
@@ -2926,7 +2296,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="101" customHeight="1" spans="1:6">
+    <row r="101" spans="1:6" ht="15.75" customHeight="1">
       <c r="A101" s="5">
         <v>50358</v>
       </c>
@@ -2940,7 +2310,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="102" customHeight="1" spans="1:6">
+    <row r="102" spans="1:6" ht="15.75" customHeight="1">
       <c r="A102" s="5">
         <v>500401</v>
       </c>
@@ -2954,7 +2324,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="103" customHeight="1" spans="1:6">
+    <row r="103" spans="1:6" ht="15.75" customHeight="1">
       <c r="A103" s="5">
         <v>500402</v>
       </c>
@@ -2968,7 +2338,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="104" customHeight="1" spans="1:6">
+    <row r="104" spans="1:6" ht="15.75" customHeight="1">
       <c r="A104" s="5">
         <v>500404</v>
       </c>
@@ -2982,7 +2352,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="105" customHeight="1" spans="1:6">
+    <row r="105" spans="1:6" ht="15.75" customHeight="1">
       <c r="A105" s="5">
         <v>50166</v>
       </c>
@@ -2996,7 +2366,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="106" customHeight="1" spans="1:6">
+    <row r="106" spans="1:6" ht="15.75" customHeight="1">
       <c r="A106" s="5">
         <v>50220</v>
       </c>
@@ -3010,7 +2380,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="107" customHeight="1" spans="1:6">
+    <row r="107" spans="1:6" ht="15.75" customHeight="1">
       <c r="A107" s="5">
         <v>25035</v>
       </c>
@@ -3027,7 +2397,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="108" customHeight="1" spans="1:6">
+    <row r="108" spans="1:6" ht="15.75" customHeight="1">
       <c r="A108" s="5">
         <v>25048</v>
       </c>
@@ -3041,7 +2411,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="109" customHeight="1" spans="1:6">
+    <row r="109" spans="1:6" ht="15.75" customHeight="1">
       <c r="A109" s="5">
         <v>25049</v>
       </c>
@@ -3055,7 +2425,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="110" customHeight="1" spans="1:6">
+    <row r="110" spans="1:6" ht="15.75" customHeight="1">
       <c r="A110" s="5">
         <v>25052</v>
       </c>
@@ -3069,7 +2439,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="111" customHeight="1" spans="1:6">
+    <row r="111" spans="1:6" ht="15.75" customHeight="1">
       <c r="A111" s="5">
         <v>25055</v>
       </c>
@@ -3083,7 +2453,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="112" customHeight="1" spans="1:6">
+    <row r="112" spans="1:6" ht="15.75" customHeight="1">
       <c r="A112" s="5">
         <v>25056</v>
       </c>
@@ -3097,7 +2467,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="113" customHeight="1" spans="1:6">
+    <row r="113" spans="1:6" ht="15.75" customHeight="1">
       <c r="A113" s="5">
         <v>25061</v>
       </c>
@@ -3111,7 +2481,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="114" customHeight="1" spans="1:6">
+    <row r="114" spans="1:6" ht="15.75" customHeight="1">
       <c r="A114" s="5">
         <v>50033</v>
       </c>
@@ -3125,7 +2495,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="115" customHeight="1" spans="1:6">
+    <row r="115" spans="1:6" ht="15.75" customHeight="1">
       <c r="A115" s="5">
         <v>50052</v>
       </c>
@@ -3139,7 +2509,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="116" customHeight="1" spans="1:6">
+    <row r="116" spans="1:6" ht="15.75" customHeight="1">
       <c r="A116" s="5">
         <v>50063</v>
       </c>
@@ -3153,7 +2523,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="117" customHeight="1" spans="1:6">
+    <row r="117" spans="1:6" ht="15.75" customHeight="1">
       <c r="A117" s="5">
         <v>50069</v>
       </c>
@@ -3170,7 +2540,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="118" customHeight="1" spans="1:6">
+    <row r="118" spans="1:6" ht="15.75" customHeight="1">
       <c r="A118" s="5">
         <v>50192</v>
       </c>
@@ -3184,7 +2554,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="119" customHeight="1" spans="1:6">
+    <row r="119" spans="1:6" ht="15.75" customHeight="1">
       <c r="A119" s="5">
         <v>50252</v>
       </c>
@@ -3198,7 +2568,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="120" customHeight="1" spans="1:6">
+    <row r="120" spans="1:6" ht="15.75" customHeight="1">
       <c r="A120" s="5">
         <v>50303</v>
       </c>
@@ -3212,7 +2582,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="121" customHeight="1" spans="1:6">
+    <row r="121" spans="1:6" ht="15.75" customHeight="1">
       <c r="A121" s="5">
         <v>50304</v>
       </c>
@@ -3226,7 +2596,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="122" customHeight="1" spans="1:6">
+    <row r="122" spans="1:6" ht="15.75" customHeight="1">
       <c r="A122" s="5">
         <v>50305</v>
       </c>
@@ -3240,7 +2610,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="123" customHeight="1" spans="1:6">
+    <row r="123" spans="1:6" ht="15.75" customHeight="1">
       <c r="A123" s="5">
         <v>50307</v>
       </c>
@@ -3254,7 +2624,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="124" customHeight="1" spans="1:6">
+    <row r="124" spans="1:6" ht="15.75" customHeight="1">
       <c r="A124" s="5">
         <v>50322</v>
       </c>
@@ -3268,7 +2638,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="125" customHeight="1" spans="1:6">
+    <row r="125" spans="1:6" ht="15.75" customHeight="1">
       <c r="A125" s="5">
         <v>50364</v>
       </c>
@@ -3282,7 +2652,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="126" customHeight="1" spans="1:6">
+    <row r="126" spans="1:6" ht="15.75" customHeight="1">
       <c r="A126" s="5">
         <v>50380</v>
       </c>
@@ -3296,7 +2666,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="127" customHeight="1" spans="1:6">
+    <row r="127" spans="1:6" ht="15.75" customHeight="1">
       <c r="A127" s="5">
         <v>50381</v>
       </c>
@@ -3310,7 +2680,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="128" customHeight="1" spans="1:6">
+    <row r="128" spans="1:6" ht="15.75" customHeight="1">
       <c r="A128" s="5">
         <v>5007</v>
       </c>
@@ -3324,7 +2694,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="129" customHeight="1" spans="1:6">
+    <row r="129" spans="1:6" ht="15.75" customHeight="1">
       <c r="A129" s="5">
         <v>25016</v>
       </c>
@@ -3338,7 +2708,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="130" customHeight="1" spans="1:6">
+    <row r="130" spans="1:6" ht="15.75" customHeight="1">
       <c r="A130" s="5">
         <v>25022</v>
       </c>
@@ -3352,7 +2722,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="131" customHeight="1" spans="1:6">
+    <row r="131" spans="1:6" ht="15.75" customHeight="1">
       <c r="A131" s="5">
         <v>25033</v>
       </c>
@@ -3366,7 +2736,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="132" customHeight="1" spans="1:6">
+    <row r="132" spans="1:6" ht="15.75" customHeight="1">
       <c r="A132" s="5">
         <v>25047</v>
       </c>
@@ -3380,7 +2750,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="133" customHeight="1" spans="1:6">
+    <row r="133" spans="1:6" ht="15.75" customHeight="1">
       <c r="A133" s="5">
         <v>25066</v>
       </c>
@@ -3394,7 +2764,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="134" customHeight="1" spans="1:6">
+    <row r="134" spans="1:6" ht="15.75" customHeight="1">
       <c r="A134" s="5">
         <v>25067</v>
       </c>
@@ -3408,7 +2778,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="135" customHeight="1" spans="1:6">
+    <row r="135" spans="1:6" ht="15.75" customHeight="1">
       <c r="A135" s="5">
         <v>50289</v>
       </c>
@@ -3422,7 +2792,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="136" customHeight="1" spans="1:6">
+    <row r="136" spans="1:6" ht="15.75" customHeight="1">
       <c r="A136" s="5">
         <v>50291</v>
       </c>
@@ -3436,7 +2806,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="137" customHeight="1" spans="1:6">
+    <row r="137" spans="1:6" ht="15.75" customHeight="1">
       <c r="A137" s="5">
         <v>50295</v>
       </c>
@@ -3450,7 +2820,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="138" customHeight="1" spans="1:6">
+    <row r="138" spans="1:6" ht="15.75" customHeight="1">
       <c r="A138" s="5">
         <v>50320</v>
       </c>
@@ -3464,7 +2834,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="139" customHeight="1" spans="1:6">
+    <row r="139" spans="1:6" ht="15.75" customHeight="1">
       <c r="A139" s="5">
         <v>50365</v>
       </c>
@@ -3478,7 +2848,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="140" customHeight="1" spans="1:6">
+    <row r="140" spans="1:6" ht="15.75" customHeight="1">
       <c r="A140" s="5">
         <v>50366</v>
       </c>
@@ -3492,7 +2862,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="141" customHeight="1" spans="1:6">
+    <row r="141" spans="1:6" ht="15.75" customHeight="1">
       <c r="A141" s="5">
         <v>50367</v>
       </c>
@@ -3506,7 +2876,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="142" customHeight="1" spans="1:6">
+    <row r="142" spans="1:6" ht="15.75" customHeight="1">
       <c r="A142" s="5">
         <v>50374</v>
       </c>
@@ -3520,7 +2890,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="143" customHeight="1" spans="1:6">
+    <row r="143" spans="1:6" ht="15.75" customHeight="1">
       <c r="A143" s="5">
         <v>500400</v>
       </c>
@@ -3534,7 +2904,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="144" customHeight="1" spans="1:6">
+    <row r="144" spans="1:6" ht="15.75" customHeight="1">
       <c r="A144" s="5">
         <v>500403</v>
       </c>
@@ -3548,7 +2918,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="145" customHeight="1" spans="1:6">
+    <row r="145" spans="1:6" ht="15.75" customHeight="1">
       <c r="A145" s="5">
         <v>25023</v>
       </c>
@@ -3562,7 +2932,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="146" customHeight="1" spans="1:6">
+    <row r="146" spans="1:6" ht="15.75" customHeight="1">
       <c r="A146" s="5">
         <v>50003</v>
       </c>
@@ -3576,7 +2946,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="147" customHeight="1" spans="1:6">
+    <row r="147" spans="1:6" ht="15.75" customHeight="1">
       <c r="A147" s="5">
         <v>50044</v>
       </c>
@@ -3590,7 +2960,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="148" customHeight="1" spans="1:6">
+    <row r="148" spans="1:6" ht="15.75" customHeight="1">
       <c r="A148" s="5">
         <v>50208</v>
       </c>
@@ -3601,12 +2971,25 @@
         <v>169</v>
       </c>
       <c r="F148" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A149" s="5">
+        <v>25051</v>
+      </c>
+      <c r="B149" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="D149" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="F149" t="s">
         <v>10</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>